<commit_message>
Refine adesanym notes and make annotation instructions self-sufficient
</commit_message>
<xml_diff>
--- a/annotation/excel/adesanym_annotation.xlsx
+++ b/annotation/excel/adesanym_annotation.xlsx
@@ -543,7 +543,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order (scores C/A/R/I/S=0/0/0/2/2).</t>
+          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/0/2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT, SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1831,7 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order (scores C/A/R/I/S=0/0/0/2/2).</t>
+          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/0/2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2415,7 @@
       <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -2867,7 +2867,7 @@
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -3091,7 +3091,7 @@
       <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/4/0/4).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/0/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3363,7 @@
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       <c r="I65" s="2" t="inlineStr"/>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3503,7 @@
       <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/0/0).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       <c r="I71" s="2" t="inlineStr"/>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/4/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3739,7 @@
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=4/0/0/0/4).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -3923,7 +3923,7 @@
       <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -4015,7 +4015,7 @@
       <c r="I78" s="2" t="inlineStr"/>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -4063,7 +4063,7 @@
       <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
       <c r="I82" s="2" t="inlineStr"/>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order (scores C/A/R/I/S=0/0/0/2/2).</t>
+          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       <c r="I83" s="2" t="inlineStr"/>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -4295,7 +4295,7 @@
       <c r="I84" s="2" t="inlineStr"/>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       <c r="I87" s="2" t="inlineStr"/>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -4523,7 +4523,7 @@
       <c r="I89" s="2" t="inlineStr"/>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4571,7 @@
       <c r="I90" s="2" t="inlineStr"/>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       <c r="I91" s="2" t="inlineStr"/>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/0).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       <c r="I94" s="2" t="inlineStr"/>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -4803,7 +4803,7 @@
       <c r="I95" s="2" t="inlineStr"/>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       <c r="I99" s="2" t="inlineStr"/>
       <c r="J99" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -5031,7 +5031,7 @@
       <c r="I100" s="2" t="inlineStr"/>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -5079,7 +5079,7 @@
       <c r="I101" s="2" t="inlineStr"/>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -5171,7 +5171,7 @@
       <c r="I103" s="2" t="inlineStr"/>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5351,7 @@
       <c r="I107" s="2" t="inlineStr"/>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/0/2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -5575,7 +5575,7 @@
       <c r="I112" s="2" t="inlineStr"/>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -5711,7 +5711,7 @@
       <c r="I115" s="2" t="inlineStr"/>
       <c r="J115" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/0/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -5759,7 +5759,7 @@
       <c r="I116" s="2" t="inlineStr"/>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -5851,7 +5851,7 @@
       <c r="I118" s="2" t="inlineStr"/>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -5899,7 +5899,7 @@
       <c r="I119" s="2" t="inlineStr"/>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -6211,7 +6211,7 @@
       <c r="I126" s="2" t="inlineStr"/>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6303,7 @@
       <c r="I128" s="2" t="inlineStr"/>
       <c r="J128" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -6395,7 +6395,7 @@
       <c r="I130" s="2" t="inlineStr"/>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/0).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -6443,7 +6443,7 @@
       <c r="I131" s="2" t="inlineStr"/>
       <c r="J131" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -6491,7 +6491,7 @@
       <c r="I132" s="2" t="inlineStr"/>
       <c r="J132" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -6583,7 +6583,7 @@
       <c r="I134" s="2" t="inlineStr"/>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -6675,7 +6675,7 @@
       <c r="I136" s="2" t="inlineStr"/>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/2/2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -6899,7 +6899,7 @@
       <c r="I141" s="2" t="inlineStr"/>
       <c r="J141" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -6991,7 +6991,7 @@
       <c r="I143" s="2" t="inlineStr"/>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -7039,7 +7039,7 @@
       <c r="I144" s="2" t="inlineStr"/>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -7131,7 +7131,7 @@
       <c r="I146" s="2" t="inlineStr"/>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order (scores C/A/R/I/S=0/0/0/2/2).</t>
+          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7223,7 @@
       <c r="I148" s="2" t="inlineStr"/>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -7315,7 +7315,7 @@
       <c r="I150" s="2" t="inlineStr"/>
       <c r="J150" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -7407,7 +7407,7 @@
       <c r="I152" s="2" t="inlineStr"/>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=4/0/4/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -7455,7 +7455,7 @@
       <c r="I153" s="2" t="inlineStr"/>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -7547,7 +7547,7 @@
       <c r="I155" s="2" t="inlineStr"/>
       <c r="J155" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -7639,7 +7639,7 @@
       <c r="I157" s="2" t="inlineStr"/>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/0).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -8171,7 +8171,7 @@
       <c r="I169" s="2" t="inlineStr"/>
       <c r="J169" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/0).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -8351,7 +8351,7 @@
       <c r="I173" s="2" t="inlineStr"/>
       <c r="J173" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -8575,7 +8575,7 @@
       <c r="I178" s="2" t="inlineStr"/>
       <c r="J178" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -8711,7 +8711,7 @@
       <c r="I181" s="2" t="inlineStr"/>
       <c r="J181" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -9067,7 +9067,7 @@
       <c r="I189" s="2" t="inlineStr"/>
       <c r="J189" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order (scores C/A/R/I/S=0/0/0/2/2).</t>
+          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -9159,7 +9159,7 @@
       <c r="I191" s="2" t="inlineStr"/>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=4/0/4/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -9251,7 +9251,7 @@
       <c r="I193" s="2" t="inlineStr"/>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -9299,7 +9299,7 @@
       <c r="I194" s="2" t="inlineStr"/>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order (scores C/A/R/I/S=0/0/0/2/2).</t>
+          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -9435,7 +9435,7 @@
       <c r="I197" s="2" t="inlineStr"/>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -9483,7 +9483,7 @@
       <c r="I198" s="2" t="inlineStr"/>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected SOCIAL via tie break order (scores C/A/R/I/S=0/0/2/2/4).</t>
+          <t>Ambiguous mixed intent; selected SOCIAL via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -9531,7 +9531,7 @@
       <c r="I199" s="2" t="inlineStr"/>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -9579,7 +9579,7 @@
       <c r="I200" s="2" t="inlineStr"/>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -9671,7 +9671,7 @@
       <c r="I202" s="2" t="inlineStr"/>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/2/2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -9807,7 +9807,7 @@
       <c r="I205" s="2" t="inlineStr"/>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -9855,7 +9855,7 @@
       <c r="I206" s="2" t="inlineStr"/>
       <c r="J206" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -10079,7 +10079,7 @@
       <c r="I211" s="2" t="inlineStr"/>
       <c r="J211" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -10127,7 +10127,7 @@
       <c r="I212" s="2" t="inlineStr"/>
       <c r="J212" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order (scores C/A/R/I/S=0/0/0/2/2).</t>
+          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -10175,7 +10175,7 @@
       <c r="I213" s="2" t="inlineStr"/>
       <c r="J213" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -10487,7 +10487,7 @@
       <c r="I220" s="2" t="inlineStr"/>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=4/0/4/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -10535,7 +10535,7 @@
       <c r="I221" s="2" t="inlineStr"/>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -10583,7 +10583,7 @@
       <c r="I222" s="2" t="inlineStr"/>
       <c r="J222" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -10631,7 +10631,7 @@
       <c r="I223" s="2" t="inlineStr"/>
       <c r="J223" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -10767,7 +10767,7 @@
       <c r="I226" s="2" t="inlineStr"/>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -10903,7 +10903,7 @@
       <c r="I229" s="2" t="inlineStr"/>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/0).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -11039,7 +11039,7 @@
       <c r="I232" s="2" t="inlineStr"/>
       <c r="J232" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -11087,7 +11087,7 @@
       <c r="I233" s="2" t="inlineStr"/>
       <c r="J233" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -11311,7 +11311,7 @@
       <c r="I238" s="2" t="inlineStr"/>
       <c r="J238" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -11403,7 +11403,7 @@
       <c r="I240" s="2" t="inlineStr"/>
       <c r="J240" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=3/0/4/0/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CORRECT_CLARIFY.</t>
         </is>
       </c>
     </row>
@@ -11495,7 +11495,7 @@
       <c r="I242" s="2" t="inlineStr"/>
       <c r="J242" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -11631,7 +11631,7 @@
       <c r="I245" s="2" t="inlineStr"/>
       <c r="J245" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -11723,7 +11723,7 @@
       <c r="I247" s="2" t="inlineStr"/>
       <c r="J247" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/0/2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -11771,7 +11771,7 @@
       <c r="I248" s="2" t="inlineStr"/>
       <c r="J248" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -11995,7 +11995,7 @@
       <c r="I253" s="2" t="inlineStr"/>
       <c r="J253" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -12043,7 +12043,7 @@
       <c r="I254" s="2" t="inlineStr"/>
       <c r="J254" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/4/0/4).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -12091,7 +12091,7 @@
       <c r="I255" s="2" t="inlineStr"/>
       <c r="J255" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=4/0/4/0/4).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: REQUEST, SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -12139,7 +12139,7 @@
       <c r="I256" s="2" t="inlineStr"/>
       <c r="J256" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -12187,7 +12187,7 @@
       <c r="I257" s="2" t="inlineStr"/>
       <c r="J257" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -12323,7 +12323,7 @@
       <c r="I260" s="2" t="inlineStr"/>
       <c r="J260" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=4/0/0/2/4).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -12371,7 +12371,7 @@
       <c r="I261" s="2" t="inlineStr"/>
       <c r="J261" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -12463,7 +12463,7 @@
       <c r="I263" s="2" t="inlineStr"/>
       <c r="J263" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/4/0/4).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -12511,7 +12511,7 @@
       <c r="I264" s="2" t="inlineStr"/>
       <c r="J264" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/0/2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -12559,7 +12559,7 @@
       <c r="I265" s="2" t="inlineStr"/>
       <c r="J265" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -12607,7 +12607,7 @@
       <c r="I266" s="2" t="inlineStr"/>
       <c r="J266" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -12699,7 +12699,7 @@
       <c r="I268" s="2" t="inlineStr"/>
       <c r="J268" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/0).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -12791,7 +12791,7 @@
       <c r="I270" s="2" t="inlineStr"/>
       <c r="J270" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -12927,7 +12927,7 @@
       <c r="I273" s="2" t="inlineStr"/>
       <c r="J273" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -12975,7 +12975,7 @@
       <c r="I274" s="2" t="inlineStr"/>
       <c r="J274" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -13023,7 +13023,7 @@
       <c r="I275" s="2" t="inlineStr"/>
       <c r="J275" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -13071,7 +13071,7 @@
       <c r="I276" s="2" t="inlineStr"/>
       <c r="J276" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -13163,7 +13163,7 @@
       <c r="I278" s="2" t="inlineStr"/>
       <c r="J278" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -13343,7 +13343,7 @@
       <c r="I282" s="2" t="inlineStr"/>
       <c r="J282" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=4/0/4/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -13655,7 +13655,7 @@
       <c r="I289" s="2" t="inlineStr"/>
       <c r="J289" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -13791,7 +13791,7 @@
       <c r="I292" s="2" t="inlineStr"/>
       <c r="J292" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -13883,7 +13883,7 @@
       <c r="I294" s="2" t="inlineStr"/>
       <c r="J294" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -14019,7 +14019,7 @@
       <c r="I297" s="2" t="inlineStr"/>
       <c r="J297" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -14155,7 +14155,7 @@
       <c r="I300" s="2" t="inlineStr"/>
       <c r="J300" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -14203,7 +14203,7 @@
       <c r="I301" s="2" t="inlineStr"/>
       <c r="J301" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/4/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -14295,7 +14295,7 @@
       <c r="I303" s="2" t="inlineStr"/>
       <c r="J303" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -14343,7 +14343,7 @@
       <c r="I304" s="2" t="inlineStr"/>
       <c r="J304" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -14391,7 +14391,7 @@
       <c r="I305" s="2" t="inlineStr"/>
       <c r="J305" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -14439,7 +14439,7 @@
       <c r="I306" s="2" t="inlineStr"/>
       <c r="J306" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -14487,7 +14487,7 @@
       <c r="I307" s="2" t="inlineStr"/>
       <c r="J307" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -14623,7 +14623,7 @@
       <c r="I310" s="2" t="inlineStr"/>
       <c r="J310" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/0/2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -14671,7 +14671,7 @@
       <c r="I311" s="2" t="inlineStr"/>
       <c r="J311" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/2/4).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -14895,7 +14895,7 @@
       <c r="I316" s="2" t="inlineStr"/>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -15119,7 +15119,7 @@
       <c r="I321" s="2" t="inlineStr"/>
       <c r="J321" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -15211,7 +15211,7 @@
       <c r="I323" s="2" t="inlineStr"/>
       <c r="J323" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/0/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -15303,7 +15303,7 @@
       <c r="I325" s="2" t="inlineStr"/>
       <c r="J325" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/0).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -15351,7 +15351,7 @@
       <c r="I326" s="2" t="inlineStr"/>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
       <c r="I327" s="2" t="inlineStr"/>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -15491,7 +15491,7 @@
       <c r="I329" s="2" t="inlineStr"/>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -15539,7 +15539,7 @@
       <c r="I330" s="2" t="inlineStr"/>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order (scores C/A/R/I/S=0/0/0/2/2).</t>
+          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -15587,7 +15587,7 @@
       <c r="I331" s="2" t="inlineStr"/>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -15679,7 +15679,7 @@
       <c r="I333" s="2" t="inlineStr"/>
       <c r="J333" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/0).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -15903,7 +15903,7 @@
       <c r="I338" s="2" t="inlineStr"/>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -15951,7 +15951,7 @@
       <c r="I339" s="2" t="inlineStr"/>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=3/0/4/2/2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CORRECT_CLARIFY.</t>
         </is>
       </c>
     </row>
@@ -16087,7 +16087,7 @@
       <c r="I342" s="2" t="inlineStr"/>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT, SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -16135,7 +16135,7 @@
       <c r="I343" s="2" t="inlineStr"/>
       <c r="J343" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -16183,7 +16183,7 @@
       <c r="I344" s="2" t="inlineStr"/>
       <c r="J344" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -16231,7 +16231,7 @@
       <c r="I345" s="2" t="inlineStr"/>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -16279,7 +16279,7 @@
       <c r="I346" s="2" t="inlineStr"/>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/0/2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -16327,7 +16327,7 @@
       <c r="I347" s="2" t="inlineStr"/>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/0).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -16463,7 +16463,7 @@
       <c r="I350" s="2" t="inlineStr"/>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -16790,7 +16790,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=4/0/4/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -16890,7 +16890,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/2/4/0/2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -16942,7 +16942,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -17042,7 +17042,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST.</t>
         </is>
       </c>
     </row>
@@ -17142,7 +17142,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -17194,7 +17194,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/0/2/0).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -17246,7 +17246,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/0).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -17490,7 +17490,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order (scores C/A/R/I/S=0/2/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected CONFIRM_ACCEPT via tie break order. Also considered: REQUEST, INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -17638,7 +17638,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order (scores C/A/R/I/S=0/0/0/2/2).</t>
+          <t>Ambiguous mixed intent; selected INFORM_CONSTRAINT via tie break order. Also considered: SOCIAL.</t>
         </is>
       </c>
     </row>
@@ -17834,7 +17834,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>
@@ -18078,7 +18078,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected REQUEST via tie break order (scores C/A/R/I/S=0/0/2/2/-2).</t>
+          <t>Ambiguous mixed intent; selected REQUEST via tie break order. Also considered: INFORM_CONSTRAINT.</t>
         </is>
       </c>
     </row>
@@ -18178,7 +18178,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order (scores C/A/R/I/S=0/0/0/0/-2).</t>
+          <t>Ambiguous mixed intent; selected CORRECT_CLARIFY via tie break order. Also considered: CONFIRM_ACCEPT.</t>
         </is>
       </c>
     </row>

</xml_diff>